<commit_message>
fix: nombres invertidos F1-6/F1-7 no llegaban completos a 1_lecturas
El override de padron traia el VALOR_NUEVO truncado (solo apellido).
Ademas, proponer_sincronizacion.py comparaba la clave sticky de un
RENAME sin el nombre, asi que un segundo cambio de nombre en el mismo
lote se confundia con el rename anterior ya aplicado y quedaba
ignorado. Se agrega NOMBRE_PADRON/NOMBRE_OPERARIO a la clave sticky.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_lecturas/inputs/registro_operario_acumulado.xlsx
+++ b/1_lecturas/inputs/registro_operario_acumulado.xlsx
@@ -5263,7 +5263,7 @@
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t>RODRIGO SAAVEDRA TRUJILLO</t>
+          <t>RODRIGO TRUJILLO SAAVEDRA</t>
         </is>
       </c>
       <c r="D141" s="7" t="n"/>
@@ -9277,7 +9277,7 @@
       </c>
       <c r="C261" s="8" t="inlineStr">
         <is>
-          <t>IGLESIA EVANGELICA BAUTISTA</t>
+          <t>RAMON REQUEZ MENDOZA</t>
         </is>
       </c>
       <c r="D261" s="7" t="n"/>
@@ -18499,7 +18499,7 @@
       </c>
       <c r="C539" s="8" t="inlineStr">
         <is>
-          <t>EFRAIN CANDACHO HUARAC</t>
+          <t>CESAR ALFREDO VIRU GASPAR</t>
         </is>
       </c>
       <c r="D539" s="7" t="n"/>
@@ -18533,7 +18533,7 @@
       </c>
       <c r="C540" s="8" t="inlineStr">
         <is>
-          <t>CESAR ALFREDO VIRU GASPAR</t>
+          <t>EFRAIN CANDACHO HUARAC</t>
         </is>
       </c>
       <c r="D540" s="7" t="n"/>

</xml_diff>